<commit_message>
Added 2 more graphs
</commit_message>
<xml_diff>
--- a/code/some_benchmarks/more_benchmarks_xlsx.xlsx
+++ b/code/some_benchmarks/more_benchmarks_xlsx.xlsx
@@ -1687,11 +1687,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="43377961"/>
-        <c:axId val="49897270"/>
+        <c:axId val="74296626"/>
+        <c:axId val="7472562"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="43377961"/>
+        <c:axId val="74296626"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1764,14 +1764,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="49897270"/>
+        <c:crossAx val="7472562"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="49897270"/>
+        <c:axId val="7472562"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1862,7 +1862,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="43377961"/>
+        <c:crossAx val="74296626"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1949,10 +1949,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.140306686110743"/>
-          <c:y val="0.163988690435142"/>
-          <c:w val="0.586283088072827"/>
-          <c:h val="0.377629129025584"/>
+          <c:x val="0.14029583146571"/>
+          <c:y val="0.164"/>
+          <c:w val="0.586239354549529"/>
+          <c:h val="0.377586206896552"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -2549,11 +2549,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="65877504"/>
-        <c:axId val="93914833"/>
+        <c:axId val="26993277"/>
+        <c:axId val="12136509"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="65877504"/>
+        <c:axId val="26993277"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2626,14 +2626,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93914833"/>
+        <c:crossAx val="12136509"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="93914833"/>
+        <c:axId val="12136509"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2724,7 +2724,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65877504"/>
+        <c:crossAx val="26993277"/>
         <c:crossesAt val="1"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2811,10 +2811,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.14027270296765"/>
-          <c:y val="0.163988690435142"/>
-          <c:w val="0.586266821138936"/>
-          <c:h val="0.377629129025584"/>
+          <c:x val="0.140284188614354"/>
+          <c:y val="0.164"/>
+          <c:w val="0.586252149515793"/>
+          <c:h val="0.377586206896552"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -3411,11 +3411,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="24854963"/>
-        <c:axId val="7723571"/>
+        <c:axId val="81623960"/>
+        <c:axId val="77889794"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="24854963"/>
+        <c:axId val="81623960"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3488,14 +3488,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="7723571"/>
+        <c:crossAx val="77889794"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="7723571"/>
+        <c:axId val="77889794"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3586,7 +3586,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="24854963"/>
+        <c:crossAx val="81623960"/>
         <c:crossesAt val="1"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -3673,10 +3673,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.140101572419182"/>
-          <c:y val="0.163962033067973"/>
-          <c:w val="0.586971383924211"/>
-          <c:h val="0.584583588487446"/>
+          <c:x val="0.140076090715944"/>
+          <c:y val="0.163974584704892"/>
+          <c:w val="0.58693611344434"/>
+          <c:h val="0.584551787491388"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -3861,11 +3861,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="54047220"/>
-        <c:axId val="42947711"/>
+        <c:axId val="94527803"/>
+        <c:axId val="42080053"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="54047220"/>
+        <c:axId val="94527803"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3938,14 +3938,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42947711"/>
+        <c:crossAx val="42080053"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="42947711"/>
+        <c:axId val="42080053"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="13"/>
@@ -4038,7 +4038,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="54047220"/>
+        <c:crossAx val="94527803"/>
         <c:crossesAt val="1"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4133,10 +4133,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.140101572419182"/>
-          <c:y val="0.163962033067973"/>
-          <c:w val="0.586971383924211"/>
-          <c:h val="0.584583588487446"/>
+          <c:x val="0.140076090715944"/>
+          <c:y val="0.163974584704892"/>
+          <c:w val="0.58693611344434"/>
+          <c:h val="0.584551787491388"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -4321,11 +4321,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="78599570"/>
-        <c:axId val="40847850"/>
+        <c:axId val="12997885"/>
+        <c:axId val="11264526"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="78599570"/>
+        <c:axId val="12997885"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4398,14 +4398,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40847850"/>
+        <c:crossAx val="11264526"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="40847850"/>
+        <c:axId val="11264526"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="13"/>
@@ -4498,7 +4498,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78599570"/>
+        <c:crossAx val="12997885"/>
         <c:crossesAt val="1"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4593,10 +4593,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.140101572419182"/>
-          <c:y val="0.163962033067973"/>
-          <c:w val="0.586971383924211"/>
-          <c:h val="0.584583588487446"/>
+          <c:x val="0.140076090715944"/>
+          <c:y val="0.163974584704892"/>
+          <c:w val="0.58693611344434"/>
+          <c:h val="0.584551787491388"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -4781,11 +4781,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="48180976"/>
-        <c:axId val="1891894"/>
+        <c:axId val="66228462"/>
+        <c:axId val="20581234"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="48180976"/>
+        <c:axId val="66228462"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4858,14 +4858,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1891894"/>
+        <c:crossAx val="20581234"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1891894"/>
+        <c:axId val="20581234"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="27"/>
@@ -4958,7 +4958,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="48180976"/>
+        <c:crossAx val="66228462"/>
         <c:crossesAt val="1"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5053,10 +5053,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.140101572419182"/>
-          <c:y val="0.163962033067973"/>
-          <c:w val="0.586971383924211"/>
-          <c:h val="0.584583588487446"/>
+          <c:x val="0.140076090715944"/>
+          <c:y val="0.163974584704892"/>
+          <c:w val="0.58693611344434"/>
+          <c:h val="0.584551787491388"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -5241,11 +5241,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="72590864"/>
-        <c:axId val="1310678"/>
+        <c:axId val="84372192"/>
+        <c:axId val="37264230"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="72590864"/>
+        <c:axId val="84372192"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5318,14 +5318,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1310678"/>
+        <c:crossAx val="37264230"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1310678"/>
+        <c:axId val="37264230"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="18"/>
@@ -5418,7 +5418,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="72590864"/>
+        <c:crossAx val="84372192"/>
         <c:crossesAt val="1"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5513,10 +5513,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.205869373345101"/>
-          <c:y val="0.148813447593935"/>
-          <c:w val="0.588316416593116"/>
-          <c:h val="0.402439024390244"/>
+          <c:x val="0.205836314847943"/>
+          <c:y val="0.148825710754017"/>
+          <c:w val="0.588271466905188"/>
+          <c:h val="0.402389781623403"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -6229,11 +6229,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="2795956"/>
-        <c:axId val="83942115"/>
+        <c:axId val="3133300"/>
+        <c:axId val="50268296"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="2795956"/>
+        <c:axId val="3133300"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6306,14 +6306,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83942115"/>
+        <c:crossAx val="50268296"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="83942115"/>
+        <c:axId val="50268296"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6378,7 +6378,7 @@
               <c:xMode val="edge"/>
               <c:yMode val="edge"/>
               <c:x val="0"/>
-              <c:y val="-8.23994726433751E-005"/>
+              <c:y val="-8.24062628759786E-005"/>
             </c:manualLayout>
           </c:layout>
           <c:overlay val="0"/>
@@ -6412,7 +6412,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2795956"/>
+        <c:crossAx val="3133300"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -7477,11 +7477,1251 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="56620011"/>
-        <c:axId val="67904899"/>
+        <c:axId val="23754559"/>
+        <c:axId val="64577963"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="56620011"/>
+        <c:axId val="23754559"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1200" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:uFill>
+                      <a:solidFill>
+                        <a:srgbClr val="ffffff"/>
+                      </a:solidFill>
+                    </a:uFill>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="0" sz="1200" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:uFill>
+                      <a:solidFill>
+                        <a:srgbClr val="ffffff"/>
+                      </a:solidFill>
+                    </a:uFill>
+                    <a:latin typeface="Arial"/>
+                  </a:rPr>
+                  <a:t>Cache sizes (number of blocks in data/instruction cache)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="b3b3b3"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1200" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:uFill>
+                  <a:solidFill>
+                    <a:srgbClr val="ffffff"/>
+                  </a:solidFill>
+                </a:uFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="64577963"/>
+        <c:crossesAt val="0"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="64577963"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="b3b3b3"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="dddddd"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:minorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1500" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:uFill>
+                      <a:solidFill>
+                        <a:srgbClr val="ffffff"/>
+                      </a:solidFill>
+                    </a:uFill>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="0" sz="1500" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:uFill>
+                      <a:solidFill>
+                        <a:srgbClr val="ffffff"/>
+                      </a:solidFill>
+                    </a:uFill>
+                    <a:latin typeface="Arial"/>
+                  </a:rPr>
+                  <a:t>Ratios</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="b3b3b3"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1200" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:uFill>
+                  <a:solidFill>
+                    <a:srgbClr val="ffffff"/>
+                  </a:solidFill>
+                </a:uFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="23754559"/>
+        <c:crossesAt val="1"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:solidFill>
+            <a:srgbClr val="b3b3b3"/>
+          </a:solidFill>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln>
+      <a:noFill/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1600" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:uFill>
+                  <a:solidFill>
+                    <a:srgbClr val="ffffff"/>
+                  </a:solidFill>
+                </a:uFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="0" sz="1600" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:uFill>
+                  <a:solidFill>
+                    <a:srgbClr val="ffffff"/>
+                  </a:solidFill>
+                </a:uFill>
+                <a:latin typeface="Arial"/>
+              </a:rPr>
+              <a:t>Blocks with n=48</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>may_2018_benchmarks!$A$158</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Primes</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="004586"/>
+            </a:solidFill>
+            <a:ln w="28800">
+              <a:solidFill>
+                <a:srgbClr val="004586"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="square"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="004586"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:dLblPos val="r"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showLeaderLines val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>may_2018_benchmarks!$F$118:$O$118</c:f>
+              <c:strCache>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>350</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>400</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v/>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>may_2018_benchmarks!$F$54:$O$54</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8.16178571428572</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8.16178571428572</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8.16178571428572</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8.16178571428572</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>8.16178571428572</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8.16178571428572</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8.16178571428572</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8.16178571428572</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v/>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>may_2018_benchmarks!$A$159</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Dijkstra</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="ff420e"/>
+            </a:solidFill>
+            <a:ln w="28800">
+              <a:solidFill>
+                <a:srgbClr val="ff420e"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="diamond"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="ff420e"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:dLblPos val="r"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showLeaderLines val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>may_2018_benchmarks!$F$118:$O$118</c:f>
+              <c:strCache>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>350</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>400</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v/>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>may_2018_benchmarks!$F$59:$O$59</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>94.6551127819549</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>51.6310526315789</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>34.21</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>32.1701503759398</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>27.591954887218</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>24.6303007518797</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>24.9739097744361</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>23.6912030075188</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v/>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>may_2018_benchmarks!$A$160</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Dijkstra w.c.</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="ffd320"/>
+            </a:solidFill>
+            <a:ln w="28800">
+              <a:solidFill>
+                <a:srgbClr val="ffd320"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="triangle"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="ffd320"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:dLblPos val="r"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showLeaderLines val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>may_2018_benchmarks!$F$118:$O$118</c:f>
+              <c:strCache>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>350</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>400</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v/>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>may_2018_benchmarks!$F$64:$O$64</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>130.239270072993</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>72.1896350364963</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>52.6297810218978</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>44.3290510948905</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>41.1465693430657</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>37.954598540146</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>35.2896350364963</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>33.6305109489051</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v/>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>may_2018_benchmarks!$A$161</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Matrix Mult</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="579d1c"/>
+            </a:solidFill>
+            <a:ln w="28800">
+              <a:solidFill>
+                <a:srgbClr val="579d1c"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="triangle"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="579d1c"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:dLblPos val="r"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showLeaderLines val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>may_2018_benchmarks!$F$118:$O$118</c:f>
+              <c:strCache>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>350</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>400</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v/>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>may_2018_benchmarks!$F$69:$N$69</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>43.3486666666667</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>34.1902051282051</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>33.6440512820513</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>33.3122564102564</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>33.2727692307692</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>33.1045641025641</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>33.1327692307692</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>32.9481538461538</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>may_2018_benchmarks!$A$162</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Determinant</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="7e0021"/>
+            </a:solidFill>
+            <a:ln w="28800">
+              <a:solidFill>
+                <a:srgbClr val="7e0021"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="triangle"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="7e0021"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:dLblPos val="r"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showLeaderLines val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>may_2018_benchmarks!$F$118:$O$118</c:f>
+              <c:strCache>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>350</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>400</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v/>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>may_2018_benchmarks!$F$79:$O$79</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>24.2793717277487</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>13.4364397905759</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>13.3338219895288</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>13.3364397905759</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>13.4416753926702</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>13.3327748691099</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>13.3327748691099</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>13.3364397905759</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v/>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>may_2018_benchmarks!$A$163</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Determinant w.c.</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="83caff"/>
+            </a:solidFill>
+            <a:ln w="28800">
+              <a:solidFill>
+                <a:srgbClr val="83caff"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="triangle"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="83caff"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:dLblPos val="r"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showLeaderLines val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>may_2018_benchmarks!$F$118:$O$118</c:f>
+              <c:strCache>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>350</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>400</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v/>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>may_2018_benchmarks!$F$74:$O$74</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>49.2428350515464</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>22.6557216494845</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>20.5959278350515</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>17.9717010309278</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>18.0490206185567</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>17.9696391752577</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>17.9696391752577</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>17.9717010309278</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v/>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="6"/>
+          <c:order val="6"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>may_2018_benchmarks!$A$164</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Hanoi</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="314004"/>
+            </a:solidFill>
+            <a:ln w="28800">
+              <a:solidFill>
+                <a:srgbClr val="314004"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="square"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="314004"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:dLblPos val="r"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showLeaderLines val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>may_2018_benchmarks!$F$118:$O$118</c:f>
+              <c:strCache>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>350</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>400</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v/>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>may_2018_benchmarks!$F$89:$O$89</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.82531052631579</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.82531052631579</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.82531052631579</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.82531052631579</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.82531052631579</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.82531052631579</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.82531052631579</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.82531052631579</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v/>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="7"/>
+          <c:order val="7"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>may_2018_benchmarks!$A$165</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Hanoi w.c.</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="aecf00"/>
+            </a:solidFill>
+            <a:ln w="28800">
+              <a:solidFill>
+                <a:srgbClr val="aecf00"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="square"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="aecf00"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:dLblPos val="r"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showLeaderLines val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>may_2018_benchmarks!$F$118:$O$118</c:f>
+              <c:strCache>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>350</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>400</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v/>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>may_2018_benchmarks!$F$84:$O$84</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v/>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>9.90709375</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5.69980208333333</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5.69980208333333</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4.73053125</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4.73053125</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>5.69980208333333</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>4.73053125</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4.73053125</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v/>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:hiLowLines>
+          <c:spPr>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:hiLowLines>
+        <c:marker val="1"/>
+        <c:axId val="44228641"/>
+        <c:axId val="59138864"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="44228641"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7554,14 +8794,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="67904899"/>
+        <c:crossAx val="59138864"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="67904899"/>
+        <c:axId val="59138864"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7652,1247 +8892,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="56620011"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:solidFill>
-            <a:srgbClr val="b3b3b3"/>
-          </a:solidFill>
-        </a:ln>
-      </c:spPr>
-    </c:plotArea>
-    <c:legend>
-      <c:legendPos val="r"/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </c:spPr>
-    </c:legend>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:srgbClr val="ffffff"/>
-    </a:solidFill>
-    <a:ln>
-      <a:noFill/>
-    </a:ln>
-  </c:spPr>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr b="0" sz="1600" spc="-1" strike="noStrike">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:uFill>
-                  <a:solidFill>
-                    <a:srgbClr val="ffffff"/>
-                  </a:solidFill>
-                </a:uFill>
-                <a:latin typeface="Arial"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr b="0" sz="1600" spc="-1" strike="noStrike">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:uFill>
-                  <a:solidFill>
-                    <a:srgbClr val="ffffff"/>
-                  </a:solidFill>
-                </a:uFill>
-                <a:latin typeface="Arial"/>
-              </a:rPr>
-              <a:t>Blocks with n=48</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:overlay val="0"/>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:lineChart>
-        <c:grouping val="standard"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>may_2018_benchmarks!$A$158</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Primes</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="004586"/>
-            </a:solidFill>
-            <a:ln w="28800">
-              <a:solidFill>
-                <a:srgbClr val="004586"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="square"/>
-            <c:size val="8"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:srgbClr val="004586"/>
-              </a:solidFill>
-            </c:spPr>
-          </c:marker>
-          <c:dLbls>
-            <c:dLblPos val="r"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="0"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showLeaderLines val="0"/>
-          </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>may_2018_benchmarks!$F$118:$O$118</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>50</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>100</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>150</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>200</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>250</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>300</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>350</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>400</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v/>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>may_2018_benchmarks!$F$54:$O$54</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>8.16178571428572</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>8.16178571428572</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>8.16178571428572</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>8.16178571428572</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>8.16178571428572</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>8.16178571428572</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>8.16178571428572</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>8.16178571428572</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v/>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>may_2018_benchmarks!$A$159</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Dijkstra</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="ff420e"/>
-            </a:solidFill>
-            <a:ln w="28800">
-              <a:solidFill>
-                <a:srgbClr val="ff420e"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="diamond"/>
-            <c:size val="8"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:srgbClr val="ff420e"/>
-              </a:solidFill>
-            </c:spPr>
-          </c:marker>
-          <c:dLbls>
-            <c:dLblPos val="r"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="0"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showLeaderLines val="0"/>
-          </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>may_2018_benchmarks!$F$118:$O$118</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>50</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>100</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>150</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>200</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>250</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>300</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>350</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>400</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v/>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>may_2018_benchmarks!$F$59:$O$59</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>94.6551127819549</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>51.6310526315789</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>34.21</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>32.1701503759398</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>27.591954887218</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>24.6303007518797</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>24.9739097744361</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>23.6912030075188</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v/>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>may_2018_benchmarks!$A$160</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Dijkstra w.c.</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="ffd320"/>
-            </a:solidFill>
-            <a:ln w="28800">
-              <a:solidFill>
-                <a:srgbClr val="ffd320"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="triangle"/>
-            <c:size val="8"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:srgbClr val="ffd320"/>
-              </a:solidFill>
-            </c:spPr>
-          </c:marker>
-          <c:dLbls>
-            <c:dLblPos val="r"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="0"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showLeaderLines val="0"/>
-          </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>may_2018_benchmarks!$F$118:$O$118</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>50</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>100</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>150</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>200</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>250</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>300</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>350</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>400</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v/>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>may_2018_benchmarks!$F$64:$O$64</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>130.239270072993</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>72.1896350364963</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>52.6297810218978</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>44.3290510948905</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>41.1465693430657</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>37.954598540146</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>35.2896350364963</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>33.6305109489051</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v/>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-        </c:ser>
-        <c:ser>
-          <c:idx val="3"/>
-          <c:order val="3"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>may_2018_benchmarks!$A$161</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Matrix Mult</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="579d1c"/>
-            </a:solidFill>
-            <a:ln w="28800">
-              <a:solidFill>
-                <a:srgbClr val="579d1c"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="triangle"/>
-            <c:size val="8"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:srgbClr val="579d1c"/>
-              </a:solidFill>
-            </c:spPr>
-          </c:marker>
-          <c:dLbls>
-            <c:dLblPos val="r"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="0"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showLeaderLines val="0"/>
-          </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>may_2018_benchmarks!$F$118:$O$118</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>50</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>100</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>150</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>200</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>250</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>300</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>350</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>400</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v/>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>may_2018_benchmarks!$F$69:$N$69</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="9"/>
-                <c:pt idx="0">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>43.3486666666667</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>34.1902051282051</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>33.6440512820513</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>33.3122564102564</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>33.2727692307692</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>33.1045641025641</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>33.1327692307692</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>32.9481538461538</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-        </c:ser>
-        <c:ser>
-          <c:idx val="4"/>
-          <c:order val="4"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>may_2018_benchmarks!$A$162</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Determinant</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="7e0021"/>
-            </a:solidFill>
-            <a:ln w="28800">
-              <a:solidFill>
-                <a:srgbClr val="7e0021"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="triangle"/>
-            <c:size val="8"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:srgbClr val="7e0021"/>
-              </a:solidFill>
-            </c:spPr>
-          </c:marker>
-          <c:dLbls>
-            <c:dLblPos val="r"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="0"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showLeaderLines val="0"/>
-          </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>may_2018_benchmarks!$F$118:$O$118</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>50</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>100</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>150</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>200</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>250</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>300</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>350</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>400</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v/>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>may_2018_benchmarks!$F$79:$O$79</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>24.2793717277487</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>13.4364397905759</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>13.3338219895288</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>13.3364397905759</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>13.4416753926702</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>13.3327748691099</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>13.3327748691099</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>13.3364397905759</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v/>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-        </c:ser>
-        <c:ser>
-          <c:idx val="5"/>
-          <c:order val="5"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>may_2018_benchmarks!$A$163</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Determinant w.c.</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="83caff"/>
-            </a:solidFill>
-            <a:ln w="28800">
-              <a:solidFill>
-                <a:srgbClr val="83caff"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="triangle"/>
-            <c:size val="8"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:srgbClr val="83caff"/>
-              </a:solidFill>
-            </c:spPr>
-          </c:marker>
-          <c:dLbls>
-            <c:dLblPos val="r"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="0"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showLeaderLines val="0"/>
-          </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>may_2018_benchmarks!$F$118:$O$118</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>50</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>100</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>150</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>200</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>250</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>300</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>350</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>400</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v/>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>may_2018_benchmarks!$F$74:$O$74</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>49.2428350515464</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>22.6557216494845</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>20.5959278350515</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>17.9717010309278</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>18.0490206185567</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>17.9696391752577</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>17.9696391752577</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>17.9717010309278</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v/>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-        </c:ser>
-        <c:ser>
-          <c:idx val="6"/>
-          <c:order val="6"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>may_2018_benchmarks!$A$164</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Hanoi</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="314004"/>
-            </a:solidFill>
-            <a:ln w="28800">
-              <a:solidFill>
-                <a:srgbClr val="314004"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="square"/>
-            <c:size val="8"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:srgbClr val="314004"/>
-              </a:solidFill>
-            </c:spPr>
-          </c:marker>
-          <c:dLbls>
-            <c:dLblPos val="r"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="0"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showLeaderLines val="0"/>
-          </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>may_2018_benchmarks!$F$118:$O$118</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>50</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>100</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>150</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>200</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>250</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>300</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>350</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>400</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v/>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>may_2018_benchmarks!$F$89:$O$89</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>1.82531052631579</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>1.82531052631579</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>1.82531052631579</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>1.82531052631579</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>1.82531052631579</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>1.82531052631579</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>1.82531052631579</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>1.82531052631579</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v/>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-        </c:ser>
-        <c:ser>
-          <c:idx val="7"/>
-          <c:order val="7"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>may_2018_benchmarks!$A$165</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Hanoi w.c.</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="aecf00"/>
-            </a:solidFill>
-            <a:ln w="28800">
-              <a:solidFill>
-                <a:srgbClr val="aecf00"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="square"/>
-            <c:size val="8"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:srgbClr val="aecf00"/>
-              </a:solidFill>
-            </c:spPr>
-          </c:marker>
-          <c:dLbls>
-            <c:dLblPos val="r"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="0"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showLeaderLines val="0"/>
-          </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>may_2018_benchmarks!$F$118:$O$118</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>50</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>100</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>150</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>200</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>250</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>300</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>350</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>400</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v/>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>may_2018_benchmarks!$F$84:$O$84</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>9.90709375</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>5.69980208333333</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>5.69980208333333</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>4.73053125</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>4.73053125</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>5.69980208333333</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>4.73053125</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>4.73053125</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v/>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-        </c:ser>
-        <c:hiLowLines>
-          <c:spPr>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-          </c:spPr>
-        </c:hiLowLines>
-        <c:marker val="1"/>
-        <c:axId val="54350354"/>
-        <c:axId val="11121424"/>
-      </c:lineChart>
-      <c:catAx>
-        <c:axId val="54350354"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="0"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr b="0" sz="900" spc="-1" strike="noStrike">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:uFill>
-                      <a:solidFill>
-                        <a:srgbClr val="ffffff"/>
-                      </a:solidFill>
-                    </a:uFill>
-                    <a:latin typeface="Arial"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr b="0" sz="900" spc="-1" strike="noStrike">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:uFill>
-                      <a:solidFill>
-                        <a:srgbClr val="ffffff"/>
-                      </a:solidFill>
-                    </a:uFill>
-                    <a:latin typeface="Arial"/>
-                  </a:rPr>
-                  <a:t>Cache sizes (number of blocks in data/instruction cache)</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-        </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:ln>
-            <a:solidFill>
-              <a:srgbClr val="b3b3b3"/>
-            </a:solidFill>
-          </a:ln>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:uFill>
-                  <a:solidFill>
-                    <a:srgbClr val="ffffff"/>
-                  </a:solidFill>
-                </a:uFill>
-                <a:latin typeface="Arial"/>
-              </a:defRPr>
-            </a:pPr>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="11121424"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="11121424"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="b3b3b3"/>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:minorGridlines>
-          <c:spPr>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="dddddd"/>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-        </c:minorGridlines>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="-5400000"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr b="0" sz="1500" spc="-1" strike="noStrike">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:uFill>
-                      <a:solidFill>
-                        <a:srgbClr val="ffffff"/>
-                      </a:solidFill>
-                    </a:uFill>
-                    <a:latin typeface="Arial"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr b="0" sz="1500" spc="-1" strike="noStrike">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:uFill>
-                      <a:solidFill>
-                        <a:srgbClr val="ffffff"/>
-                      </a:solidFill>
-                    </a:uFill>
-                    <a:latin typeface="Arial"/>
-                  </a:rPr>
-                  <a:t>Ratios</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-        </c:title>
-        <c:numFmt formatCode="General" sourceLinked="0"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:ln>
-            <a:solidFill>
-              <a:srgbClr val="b3b3b3"/>
-            </a:solidFill>
-          </a:ln>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:uFill>
-                  <a:solidFill>
-                    <a:srgbClr val="ffffff"/>
-                  </a:solidFill>
-                </a:uFill>
-                <a:latin typeface="Arial"/>
-              </a:defRPr>
-            </a:pPr>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="54350354"/>
+        <c:crossAx val="44228641"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -9957,11 +9957,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="24838278"/>
-        <c:axId val="81217402"/>
+        <c:axId val="74468881"/>
+        <c:axId val="13205211"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="24838278"/>
+        <c:axId val="74468881"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -9974,7 +9974,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr b="0" sz="900" spc="-1" strike="noStrike">
+                  <a:defRPr b="0" sz="1200" spc="-1" strike="noStrike">
                     <a:solidFill>
                       <a:srgbClr val="000000"/>
                     </a:solidFill>
@@ -9987,7 +9987,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr b="0" sz="900" spc="-1" strike="noStrike">
+                  <a:rPr b="0" sz="1200" spc="-1" strike="noStrike">
                     <a:solidFill>
                       <a:srgbClr val="000000"/>
                     </a:solidFill>
@@ -10020,7 +10020,7 @@
           <a:bodyPr/>
           <a:p>
             <a:pPr>
-              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:defRPr b="0" sz="1200" spc="-1" strike="noStrike">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
@@ -10034,14 +10034,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="81217402"/>
-        <c:crosses val="autoZero"/>
+        <c:crossAx val="13205211"/>
+        <c:crossesAt val="0"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="81217402"/>
+        <c:axId val="13205211"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -10118,7 +10118,7 @@
           <a:bodyPr/>
           <a:p>
             <a:pPr>
-              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:defRPr b="0" sz="1200" spc="-1" strike="noStrike">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
@@ -10132,8 +10132,8 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="24838278"/>
-        <c:crosses val="autoZero"/>
+        <c:crossAx val="74468881"/>
+        <c:crossesAt val="1"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:spPr>
@@ -10960,11 +10960,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="74623975"/>
-        <c:axId val="14857941"/>
+        <c:axId val="42440279"/>
+        <c:axId val="78328695"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="74623975"/>
+        <c:axId val="42440279"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11037,14 +11037,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="14857941"/>
+        <c:crossAx val="78328695"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="14857941"/>
+        <c:axId val="78328695"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11135,7 +11135,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="74623975"/>
+        <c:crossAx val="42440279"/>
         <c:crossesAt val="1"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -11222,10 +11222,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.140270834344513"/>
-          <c:y val="0.164074074074074"/>
-          <c:w val="0.586370916856768"/>
-          <c:h val="0.652314814814815"/>
+          <c:x val="0.140286177902345"/>
+          <c:y val="0.164089267524771"/>
+          <c:w val="0.586320499582043"/>
+          <c:h val="0.652282618760996"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -11582,11 +11582,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="63618162"/>
-        <c:axId val="89392977"/>
+        <c:axId val="49815441"/>
+        <c:axId val="55811892"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="63618162"/>
+        <c:axId val="49815441"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11659,14 +11659,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="89392977"/>
+        <c:crossAx val="55811892"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="89392977"/>
+        <c:axId val="55811892"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11757,7 +11757,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="63618162"/>
+        <c:crossAx val="49815441"/>
         <c:crossesAt val="1"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -11844,10 +11844,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.140280756482745"/>
-          <c:y val="0.164074074074074"/>
-          <c:w val="0.586371612400078"/>
-          <c:h val="0.652314814814815"/>
+          <c:x val="0.140257434531735"/>
+          <c:y val="0.164089267524771"/>
+          <c:w val="0.586329338659565"/>
+          <c:h val="0.652282618760996"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -12204,11 +12204,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="87132294"/>
-        <c:axId val="19884329"/>
+        <c:axId val="81638952"/>
+        <c:axId val="14715683"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="87132294"/>
+        <c:axId val="81638952"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -12281,14 +12281,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19884329"/>
+        <c:crossAx val="14715683"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="19884329"/>
+        <c:axId val="14715683"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -12379,7 +12379,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="87132294"/>
+        <c:crossAx val="81638952"/>
         <c:crossesAt val="1"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -12466,10 +12466,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.140239884012126"/>
-          <c:y val="0.163988690435142"/>
-          <c:w val="0.586265981283775"/>
-          <c:h val="0.377629129025584"/>
+          <c:x val="0.140224679188313"/>
+          <c:y val="0.164"/>
+          <c:w val="0.586252830691355"/>
+          <c:h val="0.377586206896552"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -13066,11 +13066,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="83323915"/>
-        <c:axId val="80259941"/>
+        <c:axId val="36882246"/>
+        <c:axId val="30270987"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="83323915"/>
+        <c:axId val="36882246"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13143,14 +13143,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80259941"/>
+        <c:crossAx val="30270987"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="80259941"/>
+        <c:axId val="30270987"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13241,7 +13241,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83323915"/>
+        <c:crossAx val="36882246"/>
         <c:crossesAt val="1"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -13328,10 +13328,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.140237990304099"/>
-          <c:y val="0.163988690435142"/>
-          <c:w val="0.586293521375055"/>
-          <c:h val="0.377629129025584"/>
+          <c:x val="0.140216471426663"/>
+          <c:y val="0.164"/>
+          <c:w val="0.586254509821389"/>
+          <c:h val="0.377586206896552"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -13928,11 +13928,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="41472561"/>
-        <c:axId val="51459991"/>
+        <c:axId val="39293759"/>
+        <c:axId val="32124936"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="41472561"/>
+        <c:axId val="39293759"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -14005,14 +14005,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="51459991"/>
+        <c:crossAx val="32124936"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="51459991"/>
+        <c:axId val="32124936"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -14103,7 +14103,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="41472561"/>
+        <c:crossAx val="39293759"/>
         <c:crossesAt val="1"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -14151,9 +14151,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>1363320</xdr:colOff>
+      <xdr:colOff>1362960</xdr:colOff>
       <xdr:row>142</xdr:row>
-      <xdr:rowOff>77400</xdr:rowOff>
+      <xdr:rowOff>77040</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -14161,8 +14161,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="4698720" y="20464560"/>
-        <a:ext cx="5665680" cy="3322800"/>
+        <a:off x="4641480" y="20464560"/>
+        <a:ext cx="5589000" cy="3322440"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -14181,9 +14181,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>32400</xdr:colOff>
-      <xdr:row>141</xdr:row>
-      <xdr:rowOff>135000</xdr:rowOff>
+      <xdr:colOff>1433520</xdr:colOff>
+      <xdr:row>148</xdr:row>
+      <xdr:rowOff>31320</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -14191,8 +14191,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="11522160" y="20444040"/>
-        <a:ext cx="5531400" cy="3238560"/>
+        <a:off x="11369520" y="20444040"/>
+        <a:ext cx="6856560" cy="4272840"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -14211,9 +14211,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>825840</xdr:colOff>
+      <xdr:colOff>825480</xdr:colOff>
       <xdr:row>141</xdr:row>
-      <xdr:rowOff>144000</xdr:rowOff>
+      <xdr:rowOff>143640</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -14221,8 +14221,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="19415160" y="20453040"/>
-        <a:ext cx="5546880" cy="3238560"/>
+        <a:off x="19157760" y="20453040"/>
+        <a:ext cx="5489640" cy="3238200"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -14235,15 +14235,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>30600</xdr:colOff>
+      <xdr:colOff>30960</xdr:colOff>
       <xdr:row>121</xdr:row>
-      <xdr:rowOff>156600</xdr:rowOff>
+      <xdr:rowOff>156960</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>734040</xdr:colOff>
-      <xdr:row>141</xdr:row>
-      <xdr:rowOff>144000</xdr:rowOff>
+      <xdr:colOff>2117160</xdr:colOff>
+      <xdr:row>148</xdr:row>
+      <xdr:rowOff>41040</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -14251,8 +14251,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="26538480" y="20453040"/>
-        <a:ext cx="5542200" cy="3238560"/>
+        <a:off x="26196120" y="20453400"/>
+        <a:ext cx="6858000" cy="4273200"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -14271,9 +14271,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>1666440</xdr:colOff>
+      <xdr:colOff>1666080</xdr:colOff>
       <xdr:row>172</xdr:row>
-      <xdr:rowOff>107640</xdr:rowOff>
+      <xdr:rowOff>107280</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -14281,8 +14281,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="5122080" y="24372720"/>
-        <a:ext cx="7336080" cy="4321800"/>
+        <a:off x="5064840" y="24372720"/>
+        <a:ext cx="7240320" cy="4321440"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -14306,9 +14306,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>1883160</xdr:colOff>
+      <xdr:colOff>1882800</xdr:colOff>
       <xdr:row>106</xdr:row>
-      <xdr:rowOff>19080</xdr:rowOff>
+      <xdr:rowOff>18720</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -14316,8 +14316,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="5258160" y="13985640"/>
-        <a:ext cx="7416720" cy="3887640"/>
+        <a:off x="5200920" y="13985640"/>
+        <a:ext cx="7320960" cy="3887280"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -14336,9 +14336,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>946440</xdr:colOff>
+      <xdr:colOff>946080</xdr:colOff>
       <xdr:row>106</xdr:row>
-      <xdr:rowOff>84240</xdr:rowOff>
+      <xdr:rowOff>83880</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -14346,8 +14346,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="16211160" y="14050800"/>
-        <a:ext cx="7385400" cy="3887640"/>
+        <a:off x="16001640" y="14050800"/>
+        <a:ext cx="7299360" cy="3887280"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -14366,9 +14366,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>1678680</xdr:colOff>
+      <xdr:colOff>1678320</xdr:colOff>
       <xdr:row>143</xdr:row>
-      <xdr:rowOff>18000</xdr:rowOff>
+      <xdr:rowOff>17640</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -14376,8 +14376,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="6648480" y="18666720"/>
-        <a:ext cx="8193600" cy="5220000"/>
+        <a:off x="6553440" y="18666720"/>
+        <a:ext cx="8107200" cy="5219640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -14396,9 +14396,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>1302840</xdr:colOff>
+      <xdr:colOff>1302480</xdr:colOff>
       <xdr:row>143</xdr:row>
-      <xdr:rowOff>18360</xdr:rowOff>
+      <xdr:rowOff>18000</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -14406,8 +14406,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="15784920" y="18667080"/>
-        <a:ext cx="8168040" cy="5220000"/>
+        <a:off x="15575400" y="18667080"/>
+        <a:ext cx="8082000" cy="5219640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -14426,9 +14426,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>303480</xdr:colOff>
+      <xdr:colOff>303120</xdr:colOff>
       <xdr:row>143</xdr:row>
-      <xdr:rowOff>18360</xdr:rowOff>
+      <xdr:rowOff>18000</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -14436,8 +14436,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="25285320" y="18667080"/>
-        <a:ext cx="8146080" cy="5220000"/>
+        <a:off x="24951960" y="18667080"/>
+        <a:ext cx="8031240" cy="5219640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -14456,9 +14456,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
-      <xdr:colOff>31680</xdr:colOff>
+      <xdr:colOff>31320</xdr:colOff>
       <xdr:row>143</xdr:row>
-      <xdr:rowOff>18360</xdr:rowOff>
+      <xdr:rowOff>18000</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -14466,8 +14466,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="34824600" y="18667080"/>
-        <a:ext cx="8078760" cy="5220000"/>
+        <a:off x="34376760" y="18667080"/>
+        <a:ext cx="7954920" cy="5219640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -14486,9 +14486,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>518040</xdr:colOff>
+      <xdr:colOff>517680</xdr:colOff>
       <xdr:row>177</xdr:row>
-      <xdr:rowOff>32040</xdr:rowOff>
+      <xdr:rowOff>31680</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -14496,8 +14496,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="15796440" y="24725160"/>
-        <a:ext cx="7371720" cy="4702680"/>
+        <a:off x="15586920" y="24725160"/>
+        <a:ext cx="7285680" cy="4702320"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -14516,9 +14516,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>507240</xdr:colOff>
+      <xdr:colOff>506880</xdr:colOff>
       <xdr:row>212</xdr:row>
-      <xdr:rowOff>8280</xdr:rowOff>
+      <xdr:rowOff>7920</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -14526,8 +14526,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="15785640" y="30391200"/>
-        <a:ext cx="7371720" cy="4702680"/>
+        <a:off x="15576120" y="30391200"/>
+        <a:ext cx="7285680" cy="4702320"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -14546,9 +14546,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>507240</xdr:colOff>
+      <xdr:colOff>506880</xdr:colOff>
       <xdr:row>247</xdr:row>
-      <xdr:rowOff>7200</xdr:rowOff>
+      <xdr:rowOff>6840</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -14556,8 +14556,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="15785640" y="36079560"/>
-        <a:ext cx="7371720" cy="4702680"/>
+        <a:off x="15576120" y="36079560"/>
+        <a:ext cx="7285680" cy="4702320"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -14576,9 +14576,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>540000</xdr:colOff>
+      <xdr:colOff>539640</xdr:colOff>
       <xdr:row>281</xdr:row>
-      <xdr:rowOff>16920</xdr:rowOff>
+      <xdr:rowOff>16560</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -14586,8 +14586,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="15818400" y="41616360"/>
-        <a:ext cx="7371720" cy="4702680"/>
+        <a:off x="15608880" y="41616360"/>
+        <a:ext cx="7285680" cy="4702320"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -14606,9 +14606,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>227160</xdr:colOff>
+      <xdr:colOff>226800</xdr:colOff>
       <xdr:row>171</xdr:row>
-      <xdr:rowOff>140400</xdr:rowOff>
+      <xdr:rowOff>140040</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -14616,8 +14616,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="6864840" y="24192360"/>
-        <a:ext cx="6525720" cy="4368600"/>
+        <a:off x="6769800" y="24192360"/>
+        <a:ext cx="6439320" cy="4368240"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -14638,20 +14638,20 @@
   <dimension ref="A1:S165"/>
   <sheetFormatPr defaultRowHeight="12.8"/>
   <cols>
-    <col collapsed="false" hidden="false" max="1" min="1" style="1" width="33.3418367346939"/>
-    <col collapsed="false" hidden="false" max="2" min="2" style="1" width="27.5408163265306"/>
-    <col collapsed="false" hidden="false" max="4" min="3" style="1" width="33.3418367346939"/>
-    <col collapsed="false" hidden="false" max="5" min="5" style="1" width="25.3775510204082"/>
-    <col collapsed="false" hidden="false" max="7" min="6" style="1" width="44.1428571428571"/>
-    <col collapsed="false" hidden="false" max="11" min="8" style="1" width="33.6122448979592"/>
-    <col collapsed="false" hidden="false" max="12" min="12" style="1" width="35.6377551020408"/>
-    <col collapsed="false" hidden="false" max="13" min="13" style="1" width="32.9387755102041"/>
-    <col collapsed="false" hidden="false" max="14" min="14" style="1" width="33.4795918367347"/>
-    <col collapsed="false" hidden="false" max="16" min="15" style="1" width="33.2091836734694"/>
-    <col collapsed="false" hidden="false" max="19" min="17" style="1" width="34.9642857142857"/>
-    <col collapsed="false" hidden="false" max="24" min="20" style="1" width="33.6122448979592"/>
-    <col collapsed="false" hidden="false" max="25" min="25" style="1" width="35.6377551020408"/>
-    <col collapsed="false" hidden="false" max="1025" min="26" style="1" width="10.8010204081633"/>
+    <col collapsed="false" hidden="false" max="1" min="1" style="1" width="32.8010204081633"/>
+    <col collapsed="false" hidden="false" max="2" min="2" style="1" width="27.2704081632653"/>
+    <col collapsed="false" hidden="false" max="4" min="3" style="1" width="32.8010204081633"/>
+    <col collapsed="false" hidden="false" max="5" min="5" style="1" width="25.1071428571429"/>
+    <col collapsed="false" hidden="false" max="7" min="6" style="1" width="43.6020408163265"/>
+    <col collapsed="false" hidden="false" max="11" min="8" style="1" width="33.2091836734694"/>
+    <col collapsed="false" hidden="false" max="12" min="12" style="1" width="35.0969387755102"/>
+    <col collapsed="false" hidden="false" max="13" min="13" style="1" width="32.530612244898"/>
+    <col collapsed="false" hidden="false" max="14" min="14" style="1" width="32.9387755102041"/>
+    <col collapsed="false" hidden="false" max="16" min="15" style="1" width="32.6683673469388"/>
+    <col collapsed="false" hidden="false" max="19" min="17" style="1" width="34.5561224489796"/>
+    <col collapsed="false" hidden="false" max="24" min="20" style="1" width="33.2091836734694"/>
+    <col collapsed="false" hidden="false" max="25" min="25" style="1" width="35.0969387755102"/>
+    <col collapsed="false" hidden="false" max="1025" min="26" style="1" width="10.6632653061225"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="23.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19461,20 +19461,20 @@
   <dimension ref="A1:R114"/>
   <sheetFormatPr defaultRowHeight="12.8"/>
   <cols>
-    <col collapsed="false" hidden="false" max="1" min="1" style="1" width="33.3418367346939"/>
-    <col collapsed="false" hidden="false" max="2" min="2" style="1" width="27.5408163265306"/>
-    <col collapsed="false" hidden="false" max="4" min="3" style="1" width="33.3418367346939"/>
-    <col collapsed="false" hidden="false" max="5" min="5" style="1" width="25.3775510204082"/>
-    <col collapsed="false" hidden="false" max="10" min="6" style="1" width="33.6122448979592"/>
-    <col collapsed="false" hidden="false" max="11" min="11" style="1" width="35.6377551020408"/>
-    <col collapsed="false" hidden="false" max="12" min="12" style="1" width="46.1683673469388"/>
-    <col collapsed="false" hidden="false" max="13" min="13" style="1" width="33.4795918367347"/>
-    <col collapsed="false" hidden="false" max="15" min="14" style="1" width="33.2091836734694"/>
-    <col collapsed="false" hidden="false" max="18" min="16" style="1" width="34.9642857142857"/>
-    <col collapsed="false" hidden="false" max="23" min="19" style="0" width="33.6122448979592"/>
-    <col collapsed="false" hidden="false" max="24" min="24" style="0" width="35.6377551020408"/>
-    <col collapsed="false" hidden="false" max="1019" min="25" style="1" width="10.8010204081633"/>
-    <col collapsed="false" hidden="false" max="1025" min="1020" style="0" width="8.50510204081633"/>
+    <col collapsed="false" hidden="false" max="1" min="1" style="1" width="32.8010204081633"/>
+    <col collapsed="false" hidden="false" max="2" min="2" style="1" width="27.2704081632653"/>
+    <col collapsed="false" hidden="false" max="4" min="3" style="1" width="32.8010204081633"/>
+    <col collapsed="false" hidden="false" max="5" min="5" style="1" width="25.1071428571429"/>
+    <col collapsed="false" hidden="false" max="10" min="6" style="1" width="33.2091836734694"/>
+    <col collapsed="false" hidden="false" max="11" min="11" style="1" width="35.0969387755102"/>
+    <col collapsed="false" hidden="false" max="12" min="12" style="1" width="45.6275510204082"/>
+    <col collapsed="false" hidden="false" max="13" min="13" style="1" width="32.9387755102041"/>
+    <col collapsed="false" hidden="false" max="15" min="14" style="1" width="32.6683673469388"/>
+    <col collapsed="false" hidden="false" max="18" min="16" style="1" width="34.5561224489796"/>
+    <col collapsed="false" hidden="false" max="23" min="19" style="0" width="33.2091836734694"/>
+    <col collapsed="false" hidden="false" max="24" min="24" style="0" width="35.0969387755102"/>
+    <col collapsed="false" hidden="false" max="1019" min="25" style="1" width="10.6632653061225"/>
+    <col collapsed="false" hidden="false" max="1025" min="1020" style="0" width="8.36734693877551"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>